<commit_message>
policy provisional + API deploy scaffolding + FO api meta hook
Fill policy worksheet with 임시(TBD) values for dev/deploy unblock,
add Railway Dockerfile and deploy guide, and wire FO API base via meta tag.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/기능정의서/정책_합의_워크시트.xlsx
+++ b/docs/기능정의서/정책_합의_워크시트.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,257 +445,264 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>작성일: 2026-06-02</t>
+          <t>「임시 합의 — 고객사 확정 전」 — 확정값은 임시(TBD)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>상태: 고객사(주미얀마 대사관)·운영팀 작성 대기</t>
+          <t>작성일: 2026-06-02 · 임시 갱신: 2026-06-03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>상태: 임시 합의 완료 — 고객사 최종 확정 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>근거: C안 FO/BO 시안 확정 (시안확정_C안.md), 개발자_체크리스트.md NO.463–484 및 관련 P0 정책·법무 항목</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1.1 목적</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>프로덕션 오픈 전 운영·법무·보안·콘텐츠 결정을 한 문서에 모아, 개발·인프라 착수 조건을 명확히 합니다.</t>
+          <t>1.1 목적</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>프로덕션 오픈 전 운영·법무·보안·콘텐츠 결정을 한 문서에 모아, 개발·인프라 착수 조건을 명확히 합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>프로토타입(html/C안/FO, BO 목업)에 들어간 가정값과 아직 미정인 항목을 구분해 기록합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>1.2 작성·승인</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>역할</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>담당</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>할 일</t>
+          <t>1.2 작성·승인</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>작성</t>
+          <t>역할</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>대사관 운영 담당, 헬프데스크, (필요 시) 현지 법무</t>
+          <t>담당</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>아래 표의 결정 필요 사항 검토 → 확정값·담당·일자 기입</t>
+          <t>할 일</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>기술 검토</t>
+          <t>작성</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>개발팀</t>
+          <t>대사관 운영 담당, 헬프데스크, (필요 시) 현지 법무</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>확정값이 FO/BO/API/DB에 반영 가능한지 코멘트 (비고란)</t>
+          <t>아래 표의 결정 필요 사항 검토 → 확정값·담당·일자 기입</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>기술 검토</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>확정값이 FO/BO/API/DB에 반영 가능한지 코멘트 (비고란)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>최종 승인</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>고객사 책임자(대사관)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>오픈 전 UAT·프로덕션 배포 직전 서명 또는 이메일 승인 (체크리스트 NO.392 연계)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1.3 완료 기준</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>• 체크리스트 NO.463–484 중 [-]/[p](워크시트) 항목의 확정값이 모두 채워짐</t>
+          <t>1.3 완료 기준</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>• 관련 P0 항목(응시료 콘텐츠 387, SMTP 172, OAuth 229, 개인정보 293·456–459, Feature Freeze 248 등)과 내용 불일치 없음</t>
+          <t>• 체크리스트 NO.463–484 중 [-]/[p](워크시트) 항목의 확정값이 모두 채워짐</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>• 관련 P0 항목(응시료 콘텐츠 387, SMTP 172, OAuth 229, 개인정보 293·456–459, Feature Freeze 248 등)과 내용 불일치 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>• 승인 후: 해당 행을 체크리스트에서 [x] 또는 구현 완료 시 [x]로 갱신 (개발자_체크리스트.md)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1.4 관련 문서</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>용도</t>
+          <t>1.4 관련 문서</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>개발자_체크리스트.md</t>
+          <t>문서</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NO.463–484 및 교차 참조 표</t>
+          <t>용도</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>시안확정_C안.md</t>
+          <t>개발자_체크리스트.md</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FO·BO·이메일 시안 기준</t>
+          <t>NO.463–484 및 교차 참조 표</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DB스키마_초안.md</t>
+          <t>시안확정_C안.md</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>수험번호·회차·감사 로그 테이블</t>
+          <t>FO·BO·이메일 시안 기준</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REST_API_명세_초안.md</t>
+          <t>DB스키마_초안.md</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>파일 업로드·수험번호 API</t>
+          <t>수험번호·회차·감사 로그 테이블</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>REST_API_명세_초안.md</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>파일 업로드·수험번호 API</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>배포_아키텍처.md</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>dev/prod 2환경, Feature Freeze</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>§2 표 기입 안내</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>확정값은 승인 전까지 비워 두거나 [ ]로 표시. 확정 후에는 구체적 수치·일자·URL·예/아니오를 기록합니다.</t>
+          <t>§2 표 기입 안내</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>확정값은 승인 전까지 비워 두거나 [ ]로 표시. 확정 후에는 구체적 수치·일자·URL·예/아니오를 기록합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>합의 항목 97행은 '합의항목' 시트에 수록 (섹션 §2.1–§2.14).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>다음 단계</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>다음 단계</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>본 워크시트 확정 후 → DB 마이그레이션·시드 데이터(백로그 #7), 체크리스트 감사 스크립트(#8) 실행.</t>
         </is>
@@ -720,7 +727,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="54" customWidth="1" min="4" max="4"/>
     <col width="49" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -799,9 +806,21 @@
           <t>회차별 금액 변동 여부, USD 병기·환율 안내 문구</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 50,000 MMK (USD ≈24 참고)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>체크 463, 352, 387</t>
@@ -834,9 +853,21 @@
           <t>Ⅰ·Ⅱ 동시 접수 시 각각 개별 납부 확정 여부</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 75,000 MMK (USD ≈36 참고), Ⅰ+Ⅱ 각각 개별 납부</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>체크 463</t>
@@ -865,9 +896,21 @@
           <t>대사관 수납처에서 실제 처리 절차(영수증 2장 등)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 합산 일괄 불가, 급수별 개별 수납·영수증</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
@@ -896,9 +939,21 @@
           <t>접수 기간 정의(MMT 자정 기준 등)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 100% (접수 기간 내, MMT 23:59:59 기준)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>체크 464</t>
@@ -931,9 +986,21 @@
           <t>시험일 기준 산정 방식(캘린더 day vs 영업일)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 60% (캘린더 day, 시험일 7일 전 00:00 MMT)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>체크 464</t>
@@ -962,9 +1029,21 @@
           <t>동일</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 30% (캘린더 day)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -989,9 +1068,21 @@
           <t>불가 예외(의료 등) 운영 여부</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 0% (예외 없음)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1016,9 +1107,21 @@
           <t>신청 접수 후 N일 이내 환불 완료 SLA</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 신청 접수 후 14영업일 이내</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1047,9 +1150,21 @@
           <t>위치·운영시간·연락처·계좌번호 최종본</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 대사관 지정 수납처 (계좌·시간 TBD)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>체크 353, 389</t>
@@ -1082,9 +1197,21 @@
           <t>향후 도입 검토 시점</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미사용</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1113,9 +1240,21 @@
           <t>체계 변경 필요 여부</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 13자리 체계 유지</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>DB §4.7, 체크 418–420</t>
@@ -1148,9 +1287,21 @@
           <t>타 국가 시험 확장 시 코드표</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 025 (미얀마)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>체크 467, 117</t>
@@ -1179,9 +1330,21 @@
           <t>만달레이 등 추가 지역 코드 목록</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 001 (양곤), 추가 지역 TBD</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1206,9 +1369,21 @@
           <t>동시 접수 시 7·8 각각 부여 확인</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) Ⅰ=7, Ⅱ=8</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1233,9 +1408,21 @@
           <t>제106회 등 회차별 시험장·코드 확정표</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 2자리 (01~, dev_seed 마스터)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1264,9 +1451,21 @@
           <t>동명이인·특수문자 정렬 규칙</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) name_en 오름차순, 0001~</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
           <t>체크 106</t>
@@ -1299,9 +1498,21 @@
           <t>회차별 수납 마감일 확정</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 수납 마감일 익일 일괄 부여</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>체크 105, 411</t>
@@ -1334,9 +1545,21 @@
           <t>예외 허용 여부</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 동일 시험장 강제, 예외 없음</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>체크 107, 465 [x]</t>
@@ -1361,9 +1584,21 @@
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 변경 불가</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1392,9 +1627,21 @@
           <t>탈퇴·반려·환불자 번호 공백 유지 vs 재사용</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 공백 유지 (재사용 안 함)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>체크 468, 97(환불자 번호 유지)</t>
@@ -1423,9 +1670,21 @@
           <t>연명부·ZIP에서 제외 규칙</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 번호 유지, 연명부·ZIP 제외</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1450,9 +1709,21 @@
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>확정 미노출 (0527)</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>체크 53, 412</t>
@@ -1485,9 +1756,21 @@
           <t>제106회(또는 1차 오픈 회차) 노출일·시각(MMT)</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 2026-08-01 09:00 MMT (dev_seed 제106회)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>체크 482, 110</t>
@@ -1516,9 +1799,21 @@
           <t>마이페이지 요약·수험표 안내(admit) 연동 여부</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 접수확인(mypage)만</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>admit은 topik.go.kr 안내만</t>
@@ -1551,9 +1846,21 @@
           <t>변경 권한(최고관리자만 등)</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 최고관리자만, 처리 이력 기록</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>체크 111</t>
@@ -1586,9 +1893,21 @@
           <t>노출일 전 CTA 숨김 vs 안내만</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 노출일 이후 CTA 표시</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>체크 425</t>
@@ -1621,9 +1940,21 @@
           <t>멘트 최종 문구(KO/MY/EN)</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>확정 이메일 미발송 (0527)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>체크 187, 50</t>
@@ -1656,9 +1987,21 @@
           <t>FO 노출일 공지만으로 충분한지</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>확정 이메일 미발송 (0527)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>체크 188, 109</t>
@@ -1691,9 +2034,21 @@
           <t>제외 목록 최종 확인</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 접수완료·수험번호 부여 제외, 나머지 발송</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>체크 298, 371</t>
@@ -1726,9 +2081,21 @@
           <t>KO/MY/EN 제목·본문·푸터 확정</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) C안 14종 초안 사용, 문구 TBD</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>체크 481, 189</t>
@@ -1761,9 +2128,21 @@
           <t>긴급 공지 시 SMS 도입 여부</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미사용 (이메일만)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>체크 471</t>
@@ -1796,9 +2175,21 @@
           <t>Google Cloud 프로젝트 소유 (대사관 vs 개발사)</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 프로젝트·소유 TBD</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>체크 472</t>
@@ -1831,9 +2222,21 @@
           <t>Client ID: ________________</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) TBD-DEV-GOOGLE-CLIENT-ID</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
           <t>체크 229</t>
@@ -1862,9 +2265,21 @@
           <t>Client ID: ________________</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) TBD-PROD-GOOGLE-CLIENT-ID</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1893,9 +2308,21 @@
           <t>dev: https://____________/oauth/callback</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) https://topik-myanmar.vercel.app/oauth/callback</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1924,9 +2351,21 @@
           <t>prod: https://____________/oauth/callback</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) https://topik-myanmar.vercel.app/oauth/callback</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1951,9 +2390,21 @@
           <t>앱 이름·로고·개인정보처리방침 URL</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 앱명·로고·방침 URL TBD</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1978,9 +2429,21 @@
           <t>운영 안내 문구</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 통합 차단, 안내 문구 TBD</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2009,9 +2472,21 @@
           <t>Gmail Workspace / AWS SES / SendGrid / 대사관 자체 등</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 제공자 TBD (SES/SendGrid 후보)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>체크 480</t>
@@ -2040,9 +2515,21 @@
           <t>noreply@____________ (실제 From)</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) noreply@topik-mm.local</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2067,9 +2554,21 @@
           <t>예: TOPIK Myanmar / 주미얀마대사관 TOPIK</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) TOPIK Myanmar</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2098,9 +2597,21 @@
           <t>헬프데스크 수신 주소</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) helpdesk@ TBD</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>체크 435</t>
@@ -2133,9 +2644,21 @@
           <t>DNS TXT 레코드 값·등록 담당(IT/DNS)</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미설정 (prod 오픈 전 설정)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
           <t>체크 172</t>
@@ -2168,9 +2691,21 @@
           <t>셀렉터·공개키·등록 담당</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미설정</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2199,9 +2734,21 @@
           <t>정책(none/quarantine/reject)</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미설정 (초기 none 검토)</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2230,9 +2777,21 @@
           <t>dev에서 실수 발송 방지 수신 화이트리스트</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) Mailtrap 등 테스트 전용</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>체크 230</t>
@@ -2265,9 +2824,21 @@
           <t>prod FO: https://____________</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) https://topik-myanmar.vercel.app</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
           <t>체크 201–203</t>
@@ -2296,9 +2867,21 @@
           <t>동일 도메인 /admin vs 별도 admin.____________</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 별도 admin.* (도메인 TBD)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2323,9 +2906,21 @@
           <t>prod: https://api.____________/api/v1</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) https://api.topik-mm.local — Railway 배포 후 실 URL 기록</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>REST_API_명세_초안.md</t>
@@ -2358,9 +2953,21 @@
           <t>dev FO/API URL 확정</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) FO: Vercel preview / API: localhost:3000</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>체크 204, 배포_아키텍처.md §4</t>
@@ -2391,11 +2998,19 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>☐ 예 ☐ 아니오</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
+          <t>임시(TBD) 아니오 (staging 없음)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2420,9 +3035,21 @@
           <t>dev 검색 차단·IP/Basic Auth 적용 여부</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) dev IP/Basic Auth 검토</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>배포 §7</t>
@@ -2455,9 +3082,21 @@
           <t>API/BO SSL 발급 주체</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) FO: Vercel / API: Railway 자동 SSL</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
           <t>체크 362</t>
@@ -2490,9 +3129,21 @@
           <t>기본 비밀번호·admin/admin 금지, 오픈 전 전원 교체</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) dev 시드만, prod 오픈 전 전원 교체</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
           <t>체크 276, 378, 368</t>
@@ -2525,9 +3176,21 @@
           <t>메뉴·기능별 권한 매트릭스 (수험번호 부여·연명부·ZIP 등)</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 최고/일반/조회 3등급 (매트릭스 초안)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
           <t>체크 476</t>
@@ -2562,11 +3225,19 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>☐ 예 ☐ 아니오</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
+          <t>임시(TBD) 아니오 (dev), prod 오픈 전 재검토</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
           <t>체크 478</t>
@@ -2601,11 +3272,19 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>☐ 예 ☐ 아니오</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
+          <t>임시(TBD) 아니오 (dev, IP 개방), prod 재검토</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
           <t>체크 479, 287</t>
@@ -2634,9 +3313,21 @@
           <t>관리자 세션 타임아웃(분)</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 30분</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2665,9 +3356,21 @@
           <t>적용 여부 + FO 세션 만료</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 미적용, 세션 7일</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
           <t>체크 473</t>
@@ -2700,9 +3403,21 @@
           <t>잠금 해제 절차·2FA/IP와 연계</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 5회 실패 잠금, BO 수동 해제</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
           <t>체크 297</t>
@@ -2735,9 +3450,21 @@
           <t>준거법·수탁 구조(호스팅·SMTP) 법무 메모</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) Myanmar PDPL 2021 준거</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
           <t>체크 456–458</t>
@@ -2770,9 +3497,21 @@
           <t>KO/MY/EN 최종본 + 수탁업체 명시</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) FO 목업 초안, 법무 검토 TBD</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
           <t>체크 386, 458</t>
@@ -2805,9 +3544,21 @@
           <t>탈퇴 후 즉시 삭제 vs N년 보관</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 탈퇴 후 3년</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
           <t>체크 293</t>
@@ -2840,9 +3591,21 @@
           <t>시험 종료 후 N년 (연명부·성적 연계)</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 시험 종료 후 3년</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
           <t>체크 433</t>
@@ -2875,9 +3638,21 @@
           <t>사진·게시글·감사 로그 파기 범위</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 접수 자동 취소, 사진 1년 후 파기</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
           <t>체크 82, 293</t>
@@ -2912,11 +3687,19 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>☐ 필요 ☐ 불필요</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="inlineStr"/>
+          <t>임시(TBD) 필요 — 14세 미만 가입 차단</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
           <t>체크 459</t>
@@ -2949,9 +3732,21 @@
           <t>PDPL/PIPA 요청 처리 SLA·담당</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 30일 이내 처리</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
           <t>체크 452</t>
@@ -2980,9 +3775,21 @@
           <t>여권번호 등 필드 암호화 여부</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 여권번호 필드 암호화</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
           <t>DB §1</t>
@@ -3015,9 +3822,21 @@
           <t>NIIED(국립국제교육원) 사용 허가 유무·범위</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 허가 절차 진행 TBD</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
           <t>체크 461</t>
@@ -3046,9 +3865,21 @@
           <t>상표 표기 가이드 준수</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) topik.go.kr 링크 유지</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
@@ -3073,9 +3904,21 @@
           <t>법적 표기 최종 확인</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 현행 푸터 유지, 법무 확인 TBD</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
@@ -3104,9 +3947,21 @@
           <t>prod에서 JPG만 제한 여부</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) JPEG only (prod)</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>체크 306, API §1.6</t>
@@ -3135,9 +3990,21 @@
           <t>상한·하한 변경</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) max 200KB</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
           <t>photo-upload.js</t>
@@ -3166,9 +4033,21 @@
           <t>검증 강도(픽셀 강제 vs 안내만)</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 3:4 안내 (픽셀 강제 없음)</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
@@ -3197,9 +4076,21 @@
           <t>강제 차단 vs BO 심사</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="2" t="inlineStr"/>
-      <c r="H76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 6개월 안내, BO 심사</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
           <t>체크 470</t>
@@ -3228,9 +4119,21 @@
           <t>6개월 경과 시 갱신 유도 여부</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 1회 등록 재사용, 6개월 경과 갱신 유도</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
@@ -3255,9 +4158,21 @@
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) BO 재심사 + 접수 반영</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
           <t>체크 422</t>
@@ -3290,9 +4205,21 @@
           <t>표준 코드·한글/미얀마어/영문 안내 문구</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) DB 6종 코드 사용</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
           <t>체크 469</t>
@@ -3325,9 +4252,21 @@
           <t>사진만 재제출 vs 취소 후 재접수</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
-      <c r="H80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 사진만 재제출</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
           <t>체크 423</t>
@@ -3360,9 +4299,21 @@
           <t>보관 기간·아카이브 (회차 종료 후)</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
-      <c r="H81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 1년 보관</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
           <t>체크 421, 433</t>
@@ -3391,9 +4342,21 @@
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
-      <c r="H82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) {수험번호}.jpg</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
           <t>체크 113, 169</t>
@@ -3426,9 +4389,21 @@
           <t>보존 기간(예: 3년/5년/영구)</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="2" t="inlineStr"/>
-      <c r="H83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 1년</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
           <t>체크 477, 139</t>
@@ -3457,9 +4432,21 @@
           <t>사용자 노출 여부</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
-      <c r="H84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 사용자 미노출</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
@@ -3488,9 +4475,21 @@
           <t>실제 보존 일수·스토리지</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
-      <c r="H85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 90일</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
           <t>체크 261</t>
@@ -3519,9 +4518,21 @@
           <t>보존 기간</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
-      <c r="H86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 1년</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
@@ -3546,9 +4557,21 @@
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr"/>
-      <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="2" t="inlineStr"/>
-      <c r="H87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>확정 Ⅰ+Ⅱ 동시 허용</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
           <t>체크 465 [x]</t>
@@ -3581,9 +4604,21 @@
           <t>임시 저장 보관 기간·자동 삭제</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 30일 후 자동 삭제</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
           <t>체크 466, 354</t>
@@ -3616,9 +4651,21 @@
           <t>분실 시 복구(본인확인)·관리자 열람</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-      <c r="H89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 4자리 이상 별도 비번</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
           <t>체크 474</t>
@@ -3651,9 +4698,21 @@
           <t>답변 N영업일·공개/비공개 답글</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 5영업일 이내</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
           <t>체크 475</t>
@@ -3686,9 +4745,21 @@
           <t>미입력 시 게시 금지 vs KO만 허용</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="2" t="inlineStr"/>
-      <c r="H91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) KO 필수, MY/EN 권장</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
           <t>체크 483</t>
@@ -3721,9 +4792,21 @@
           <t>개정 시 재동의 팝업/로그인 차단</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 재동의 팝업</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
           <t>체크 484</t>
@@ -3758,11 +4841,19 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>☐ 이메일만 ☐ SMS 추가</t>
-        </is>
-      </c>
-      <c r="G93" s="2" t="inlineStr"/>
-      <c r="H93" s="2" t="inlineStr"/>
+          <t>임시(TBD) 이메일만</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
           <t>체크 471</t>
@@ -3795,9 +4886,21 @@
           <t>동결 기간 예외 승인자(2인)</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="2" t="inlineStr"/>
-      <c r="H94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 접수 시작 D-3 ~ 접수 종료, 예외 2인 승인</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
           <t>체크 248, 배포_아키텍처.md §6</t>
@@ -3822,9 +4925,21 @@
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr"/>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
-      <c r="H95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 긴급 버그·보안·핫픽스 (승인制)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
@@ -3845,9 +4960,21 @@
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr"/>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr"/>
-      <c r="H96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 신규 화면·스키마·대규모 리팩터 금지</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
@@ -3876,9 +5003,21 @@
           <t>접수 시작·마감·시험일·수납 마감·수험번호 노출일 일괄표</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
-      <c r="H97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) 제106회 (dev_seed 일정)</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
           <t>체크 388, 396</t>
@@ -3911,9 +5050,21 @@
           <t>UAT 완료일·승인자</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>임시(TBD) UAT 일정·승인자 TBD</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>개발팀</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
           <t>체크 392</t>

</xml_diff>